<commit_message>
Update maintenance map (bearing to tomago added)
</commit_message>
<xml_diff>
--- a/docs/qmd/chapter_1/downloads/antenna_log.xlsx
+++ b/docs/qmd/chapter_1/downloads/antenna_log.xlsx
@@ -1133,11 +1133,11 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="H16" t="e">
-        <v>#N/A</v>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H16">
+        <v>112.2</v>
       </c>
       <c r="I16">
         <v>8</v>
@@ -1182,11 +1182,11 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>TODO</t>
-        </is>
-      </c>
-      <c r="H17" t="e">
-        <v>#N/A</v>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="H17">
+        <v>292.2</v>
       </c>
       <c r="I17">
         <v>10</v>

</xml_diff>